<commit_message>
change label for ref2 and ref 3
</commit_message>
<xml_diff>
--- a/public/consignmentapp_SampleDATA/billdata.xlsx
+++ b/public/consignmentapp_SampleDATA/billdata.xlsx
@@ -42,12 +42,6 @@
     <t xml:space="preserve"> A_Amount</t>
   </si>
   <si>
-    <t>Ref 2</t>
-  </si>
-  <si>
-    <t>Ref 3</t>
-  </si>
-  <si>
     <t>Freight Type</t>
   </si>
   <si>
@@ -118,6 +112,12 @@
   </si>
   <si>
     <t>mode</t>
+  </si>
+  <si>
+    <t>Freight PO</t>
+  </si>
+  <si>
+    <t>Freight GRN</t>
   </si>
 </sst>
 </file>
@@ -668,22 +668,22 @@
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>0</v>
@@ -710,63 +710,63 @@
         <v>7</v>
       </c>
       <c r="O1" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="R1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>11</v>
-      </c>
       <c r="S1" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="T1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="V1" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="V1" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" s="17">
         <v>5104</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E2" s="17">
         <v>5509</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H2" s="9">
         <v>2500224</v>
       </c>
       <c r="I2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="11" t="s">
         <v>13</v>
-      </c>
-      <c r="J2" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" s="11" t="s">
-        <v>15</v>
       </c>
       <c r="L2" s="12">
         <v>1315456</v>
@@ -784,7 +784,7 @@
         <v>5002981654</v>
       </c>
       <c r="Q2" s="17" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R2" s="18"/>
       <c r="S2" s="18"/>
@@ -794,22 +794,22 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B3" s="17">
         <v>5104</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E3" s="17">
         <v>5508</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G3" s="8"/>
       <c r="H3" s="9"/>
@@ -830,22 +830,22 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" s="17">
         <v>5104</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E4" s="17">
         <v>5508</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G4" s="8"/>
       <c r="H4" s="9"/>
@@ -866,22 +866,22 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="17">
         <v>5104</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E5" s="17">
         <v>5508</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G5" s="8"/>
       <c r="H5" s="9"/>
@@ -902,22 +902,22 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" s="17">
         <v>5104</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E6" s="17">
         <v>5508</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="9"/>
@@ -938,22 +938,22 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="17">
         <v>5104</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E7" s="17">
         <v>5514</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="9"/>
@@ -974,22 +974,22 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B8" s="17">
         <v>5803</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E8" s="17">
         <v>5501</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G8" s="8"/>
       <c r="H8" s="9"/>
@@ -1010,22 +1010,22 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B9" s="17">
         <v>5803</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E9" s="17">
         <v>5501</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="9"/>

</xml_diff>